<commit_message>
Osvežen build pre slanja
</commit_message>
<xml_diff>
--- a/excel rad izmenjen/sifrarnik-paket/SPC_atributivne.xlsx
+++ b/excel rad izmenjen/sifrarnik-paket/SPC_atributivne.xlsx
@@ -8303,7 +8303,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -8354,7 +8354,7 @@
         <v>5502-A</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v>G</v>
       </c>
       <c r="C2" t="str">
         <v>RN-2024-002</v>
@@ -8363,13 +8363,13 @@
         <v>Osovina</v>
       </c>
       <c r="E2" t="str">
-        <v>Kontrola kvaliteta</v>
+        <v>Merljive kontrola</v>
       </c>
       <c r="F2">
         <v>7</v>
       </c>
-      <c r="G2">
-        <v>1</v>
+      <c r="G2" t="str">
+        <v/>
       </c>
       <c r="H2">
         <v>100</v>
@@ -8381,7 +8381,7 @@
         <v>DA</v>
       </c>
       <c r="K2" t="str">
-        <v/>
+        <v>Pogon G — Masinska obrada</v>
       </c>
       <c r="L2" t="str">
         <v>deo</v>
@@ -8439,43 +8439,43 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>MRAP-001</v>
+        <v>DEMO-001</v>
       </c>
       <c r="B4" t="str">
-        <v/>
+        <v>B</v>
       </c>
       <c r="C4" t="str">
-        <v/>
+        <v>RN-2026-DEMO001</v>
       </c>
       <c r="D4" t="str">
-        <v>MRAP komplet</v>
+        <v>Test nosač — demo</v>
       </c>
       <c r="E4" t="str">
-        <v>Finalna vizuelna kontrola celog vozila</v>
-      </c>
-      <c r="F4" t="str">
-        <v>48</v>
-      </c>
-      <c r="G4" t="str">
-        <v>1</v>
-      </c>
-      <c r="H4" t="str">
-        <v>5</v>
+        <v>Laser sečenje</v>
+      </c>
+      <c r="F4">
+        <v>2</v>
+      </c>
+      <c r="G4">
+        <v>3</v>
+      </c>
+      <c r="H4">
+        <v>50</v>
       </c>
       <c r="I4" t="str">
-        <v>MRAP_SOP.jpg</v>
+        <v>DEMO-01.png</v>
       </c>
       <c r="J4" t="str">
         <v>DA</v>
       </c>
       <c r="K4" t="str">
-        <v>MRAP — oklopno vozilo</v>
+        <v>Pogon B — Preseraj</v>
       </c>
       <c r="L4" t="str">
-        <v>vozilo</v>
+        <v>deo</v>
       </c>
       <c r="M4" t="str">
-        <v>MRAP</v>
+        <v/>
       </c>
       <c r="N4" t="str">
         <v/>
@@ -8483,43 +8483,43 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>MRAP1-001</v>
+        <v>DEMO-001</v>
       </c>
       <c r="B5" t="str">
-        <v/>
+        <v>F</v>
       </c>
       <c r="C5" t="str">
-        <v/>
+        <v>RN-2026-DEMO001-F</v>
       </c>
       <c r="D5" t="str">
-        <v>MRAP1 komplet</v>
+        <v/>
       </c>
       <c r="E5" t="str">
-        <v>Finalna vizuelna kontrola celog vozila</v>
-      </c>
-      <c r="F5" t="str">
-        <v>48</v>
+        <v>Završna kontrola</v>
+      </c>
+      <c r="F5">
+        <v>6</v>
       </c>
       <c r="G5" t="str">
-        <v>1</v>
+        <v/>
       </c>
       <c r="H5" t="str">
-        <v>5</v>
+        <v/>
       </c>
       <c r="I5" t="str">
-        <v>MRAP1_SOP.jpg</v>
+        <v/>
       </c>
       <c r="J5" t="str">
         <v>DA</v>
       </c>
       <c r="K5" t="str">
-        <v>MRAP1 — oklopno vozilo 6x6</v>
+        <v>Pogon F — Završna</v>
       </c>
       <c r="L5" t="str">
-        <v>vozilo</v>
+        <v>deo</v>
       </c>
       <c r="M5" t="str">
-        <v>MRAP1</v>
+        <v/>
       </c>
       <c r="N5" t="str">
         <v/>
@@ -8527,43 +8527,43 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>NM-001</v>
+        <v>MRAP-001</v>
       </c>
       <c r="B6" t="str">
-        <v>C</v>
+        <v/>
       </c>
       <c r="C6" t="str">
-        <v>RN-2026-NM001</v>
+        <v/>
       </c>
       <c r="D6" t="str">
-        <v>Nosač motora</v>
+        <v>MRAP komplet</v>
       </c>
       <c r="E6" t="str">
-        <v>Geometrijska kontrola</v>
-      </c>
-      <c r="F6">
-        <v>3</v>
+        <v>Finalna vizuelna kontrola celog vozila</v>
+      </c>
+      <c r="F6" t="str">
+        <v>48</v>
       </c>
       <c r="G6" t="str">
-        <v/>
-      </c>
-      <c r="H6">
-        <v>100</v>
+        <v>1</v>
+      </c>
+      <c r="H6" t="str">
+        <v>5</v>
       </c>
       <c r="I6" t="str">
-        <v>NM-01.png</v>
+        <v>MRAP_SOP.jpg</v>
       </c>
       <c r="J6" t="str">
         <v>DA</v>
       </c>
       <c r="K6" t="str">
-        <v>Atributivne — Karoserija</v>
+        <v>MRAP — oklopno vozilo</v>
       </c>
       <c r="L6" t="str">
-        <v>deo</v>
+        <v>vozilo</v>
       </c>
       <c r="M6" t="str">
-        <v/>
+        <v>MRAP</v>
       </c>
       <c r="N6" t="str">
         <v/>
@@ -8571,43 +8571,43 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>NT-001</v>
+        <v>MRAP1-001</v>
       </c>
       <c r="B7" t="str">
-        <v>A</v>
+        <v/>
       </c>
       <c r="C7" t="str">
-        <v>RN-2026-NT001-A</v>
+        <v/>
       </c>
       <c r="D7" t="str">
-        <v>Nosač motora</v>
+        <v>MRAP1 komplet</v>
       </c>
       <c r="E7" t="str">
-        <v>Vizuelna kontrola ulazna</v>
-      </c>
-      <c r="F7">
+        <v>Finalna vizuelna kontrola celog vozila</v>
+      </c>
+      <c r="F7" t="str">
+        <v>48</v>
+      </c>
+      <c r="G7" t="str">
         <v>1</v>
       </c>
-      <c r="G7" t="str">
-        <v/>
-      </c>
-      <c r="H7">
-        <v>50</v>
+      <c r="H7" t="str">
+        <v>5</v>
       </c>
       <c r="I7" t="str">
-        <v>nosac motora NTV.png</v>
+        <v>MRAP1_SOP.jpg</v>
       </c>
       <c r="J7" t="str">
         <v>DA</v>
       </c>
       <c r="K7" t="str">
-        <v>Atributivne — Ulazna</v>
+        <v>MRAP1 — oklopno vozilo 6x6</v>
       </c>
       <c r="L7" t="str">
-        <v>deo</v>
+        <v>vozilo</v>
       </c>
       <c r="M7" t="str">
-        <v/>
+        <v>MRAP1</v>
       </c>
       <c r="N7" t="str">
         <v/>
@@ -8615,37 +8615,37 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>NT-001</v>
+        <v>NM-001</v>
       </c>
       <c r="B8" t="str">
-        <v>C</v>
+        <v>A</v>
       </c>
       <c r="C8" t="str">
-        <v>RN-2026-NT001-C</v>
+        <v>RN-2026-NM001</v>
       </c>
       <c r="D8" t="str">
         <v>Nosač motora</v>
       </c>
       <c r="E8" t="str">
-        <v>Zavarivanje</v>
+        <v>Vizuelna kontrola ulazna</v>
       </c>
       <c r="F8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G8" t="str">
         <v/>
       </c>
       <c r="H8">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="I8" t="str">
-        <v>nosac motora NTV.png</v>
+        <v>NM-01.png</v>
       </c>
       <c r="J8" t="str">
         <v>DA</v>
       </c>
       <c r="K8" t="str">
-        <v>Atributivne — Karoserija</v>
+        <v>Pogon A — Ulazna kontrola</v>
       </c>
       <c r="L8" t="str">
         <v>deo</v>
@@ -8659,37 +8659,37 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>NT-001</v>
+        <v>NM-001</v>
       </c>
       <c r="B9" t="str">
-        <v>F</v>
+        <v>B</v>
       </c>
       <c r="C9" t="str">
-        <v>RN-2026-NT001-F</v>
+        <v>RN-2026-NM001</v>
       </c>
       <c r="D9" t="str">
         <v>Nosač motora</v>
       </c>
       <c r="E9" t="str">
-        <v>Završna kontrola</v>
+        <v>Laser sečenje</v>
       </c>
       <c r="F9">
-        <v>6</v>
-      </c>
-      <c r="G9" t="str">
-        <v/>
+        <v>2</v>
+      </c>
+      <c r="G9">
+        <v>3</v>
       </c>
       <c r="H9">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="I9" t="str">
-        <v>nosac motora NTV.png</v>
+        <v>NM-01.png</v>
       </c>
       <c r="J9" t="str">
         <v>DA</v>
       </c>
       <c r="K9" t="str">
-        <v>Atributivne — Finalna</v>
+        <v>Pogon B — Preseraj</v>
       </c>
       <c r="L9" t="str">
         <v>deo</v>
@@ -8703,51 +8703,315 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>NTV-001</v>
+        <v>NM-001</v>
       </c>
       <c r="B10" t="str">
-        <v/>
+        <v>C</v>
       </c>
       <c r="C10" t="str">
-        <v/>
+        <v>RN-2026-NM001</v>
       </c>
       <c r="D10" t="str">
-        <v>NTV komplet</v>
+        <v>Nosač motora</v>
       </c>
       <c r="E10" t="str">
-        <v>Finalna vizuelna kontrola celog vozila</v>
-      </c>
-      <c r="F10" t="str">
-        <v>48</v>
+        <v>Geometrijska kontrola</v>
+      </c>
+      <c r="F10">
+        <v>3</v>
       </c>
       <c r="G10" t="str">
-        <v>1</v>
-      </c>
-      <c r="H10" t="str">
-        <v>5</v>
+        <v/>
+      </c>
+      <c r="H10">
+        <v>100</v>
       </c>
       <c r="I10" t="str">
-        <v>NTV_SOP.jpg</v>
+        <v>NM-01.png</v>
       </c>
       <c r="J10" t="str">
         <v>DA</v>
       </c>
       <c r="K10" t="str">
+        <v>Atributivne — Karoserija</v>
+      </c>
+      <c r="L10" t="str">
+        <v>deo</v>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
+      <c r="N10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>NM-001</v>
+      </c>
+      <c r="B11" t="str">
+        <v>F</v>
+      </c>
+      <c r="C11" t="str">
+        <v>RN-2026-NM001</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Nosač motora</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Završna kontrola</v>
+      </c>
+      <c r="F11">
+        <v>6</v>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11">
+        <v>100</v>
+      </c>
+      <c r="I11" t="str">
+        <v>NM-01.png</v>
+      </c>
+      <c r="J11" t="str">
+        <v>DA</v>
+      </c>
+      <c r="K11" t="str">
+        <v>Pogon F — Završna</v>
+      </c>
+      <c r="L11" t="str">
+        <v>deo</v>
+      </c>
+      <c r="M11" t="str">
+        <v/>
+      </c>
+      <c r="N11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>NT-001</v>
+      </c>
+      <c r="B12" t="str">
+        <v>A</v>
+      </c>
+      <c r="C12" t="str">
+        <v>RN-2026-NT001-A</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Nosač motora</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Vizuelna kontrola ulazna</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12">
+        <v>50</v>
+      </c>
+      <c r="I12" t="str">
+        <v>nosac motora NTV.png</v>
+      </c>
+      <c r="J12" t="str">
+        <v>DA</v>
+      </c>
+      <c r="K12" t="str">
+        <v>Atributivne — Ulazna</v>
+      </c>
+      <c r="L12" t="str">
+        <v>deo</v>
+      </c>
+      <c r="M12" t="str">
+        <v/>
+      </c>
+      <c r="N12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>NT-001</v>
+      </c>
+      <c r="B13" t="str">
+        <v>B</v>
+      </c>
+      <c r="C13" t="str">
+        <v>RN-2026-NT001-B</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Nosač motora</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Laser sečenje</v>
+      </c>
+      <c r="F13">
+        <v>2</v>
+      </c>
+      <c r="G13">
+        <v>3</v>
+      </c>
+      <c r="H13">
+        <v>50</v>
+      </c>
+      <c r="I13" t="str">
+        <v>nosac motora NTV.png</v>
+      </c>
+      <c r="J13" t="str">
+        <v>DA</v>
+      </c>
+      <c r="K13" t="str">
+        <v>Pogon B — Preseraj</v>
+      </c>
+      <c r="L13" t="str">
+        <v>deo</v>
+      </c>
+      <c r="M13" t="str">
+        <v/>
+      </c>
+      <c r="N13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>NT-001</v>
+      </c>
+      <c r="B14" t="str">
+        <v>C</v>
+      </c>
+      <c r="C14" t="str">
+        <v>RN-2026-NT001-C</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Nosač motora</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Zavarivanje</v>
+      </c>
+      <c r="F14">
+        <v>3</v>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14">
+        <v>50</v>
+      </c>
+      <c r="I14" t="str">
+        <v>nosac motora NTV.png</v>
+      </c>
+      <c r="J14" t="str">
+        <v>DA</v>
+      </c>
+      <c r="K14" t="str">
+        <v>Atributivne — Karoserija</v>
+      </c>
+      <c r="L14" t="str">
+        <v>deo</v>
+      </c>
+      <c r="M14" t="str">
+        <v/>
+      </c>
+      <c r="N14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>NT-001</v>
+      </c>
+      <c r="B15" t="str">
+        <v>F</v>
+      </c>
+      <c r="C15" t="str">
+        <v>RN-2026-NT001-F</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Nosač motora</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Završna kontrola</v>
+      </c>
+      <c r="F15">
+        <v>6</v>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15">
+        <v>50</v>
+      </c>
+      <c r="I15" t="str">
+        <v>nosac motora NTV.png</v>
+      </c>
+      <c r="J15" t="str">
+        <v>DA</v>
+      </c>
+      <c r="K15" t="str">
+        <v>Atributivne — Finalna</v>
+      </c>
+      <c r="L15" t="str">
+        <v>deo</v>
+      </c>
+      <c r="M15" t="str">
+        <v/>
+      </c>
+      <c r="N15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>NTV-001</v>
+      </c>
+      <c r="B16" t="str">
+        <v/>
+      </c>
+      <c r="C16" t="str">
+        <v/>
+      </c>
+      <c r="D16" t="str">
+        <v>NTV komplet</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Finalna vizuelna kontrola celog vozila</v>
+      </c>
+      <c r="F16" t="str">
+        <v>48</v>
+      </c>
+      <c r="G16" t="str">
+        <v>1</v>
+      </c>
+      <c r="H16" t="str">
+        <v>5</v>
+      </c>
+      <c r="I16" t="str">
+        <v>NTV_SOP.jpg</v>
+      </c>
+      <c r="J16" t="str">
+        <v>DA</v>
+      </c>
+      <c r="K16" t="str">
         <v>NTV — novo terensko vozilo</v>
       </c>
-      <c r="L10" t="str">
+      <c r="L16" t="str">
         <v>vozilo</v>
       </c>
-      <c r="M10" t="str">
+      <c r="M16" t="str">
         <v>NTV</v>
       </c>
-      <c r="N10" t="str">
+      <c r="N16" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N16"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>